<commit_message>
Validate Excel categories and refresh import template
</commit_message>
<xml_diff>
--- a/public/downloads/Corevity-Product-Import-Example.xlsx
+++ b/public/downloads/Corevity-Product-Import-Example.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สินค้า" sheetId="1" r:id="R2e367eea393b4750"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="วิธีใช้งาน" sheetId="2" r:id="R027e1e2dcb874291"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="สินค้า" sheetId="1" r:id="Rf94559a722f74d56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="วิธีใช้งาน" sheetId="2" r:id="Rda7c13ce9549432e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -37,6 +37,11 @@
       <x:b/>
       <x:sz val="11"/>
       <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
   <x:fills count="4">
@@ -58,12 +63,18 @@
     </x:fill>
   </x:fills>
   <x:borders count="1">
-    <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -78,7 +89,11 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -287,7 +302,7 @@
     <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
@@ -341,7 +356,7 @@
       </x:c>
       <x:c r="C2" s="5"/>
       <x:c r="D2" s="5" t="str">
-        <x:v>ลู่วิ่ง</x:v>
+        <x:v>Treadmills</x:v>
       </x:c>
       <x:c r="E2" s="5" t="str">
         <x:v>EXAMPLE-001</x:v>
@@ -374,7 +389,7 @@
       </x:c>
       <x:c r="C3" s="5"/>
       <x:c r="D3" s="5" t="str">
-        <x:v>จักรยานออกกำลังกาย</x:v>
+        <x:v>Upright Bike</x:v>
       </x:c>
       <x:c r="E3" s="5" t="str">
         <x:v>EXAMPLE-002</x:v>
@@ -407,7 +422,7 @@
       </x:c>
       <x:c r="C4" s="5"/>
       <x:c r="D4" s="5" t="str">
-        <x:v>เครื่องกรรเชียงบก</x:v>
+        <x:v>Rowwing</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
         <x:v>EXAMPLE-003</x:v>
@@ -1907,12 +1922,15 @@
       <x:c r="H201" s="10"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="I2:I201">
       <x:formula1>"พร้อมขาย,ขายแล้ว"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F201">
       <x:formula1>"Excellent,Good,Fair,Needs Repair"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D2:D201">
+      <x:formula1>INDIRECT("'วิธีใช้งาน'!$D$2:$D$25")</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1926,6 +1944,8 @@
   </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4" hidden="0" customWidth="1"/>
     <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="100" hidden="0" customWidth="1"/>
   </x:cols>
@@ -1938,7 +1958,9 @@
         <x:v>รายละเอียด</x:v>
       </x:c>
       <x:c r="C1" s="1"/>
-      <x:c r="D1" s="1"/>
+      <x:c r="D1" s="3" t="str">
+        <x:v>Category (24 หมวด)</x:v>
+      </x:c>
       <x:c r="E1" s="1"/>
       <x:c r="F1" s="1"/>
       <x:c r="G1" s="1"/>
@@ -1948,14 +1970,16 @@
       <x:c r="K1" s="1"/>
     </x:row>
     <x:row r="2" ht="35" customHeight="1">
-      <x:c r="A2" s="12" t="str">
+      <x:c r="A2" s="13" t="str">
         <x:v>ก่อนเริ่ม</x:v>
       </x:c>
       <x:c r="B2" s="11" t="str">
         <x:v>ข้อมูล 3 แถวในชีตสินค้าเป็นข้อมูลสมมติ ให้แทนที่หรือลบทิ้งก่อนนำเข้า</x:v>
       </x:c>
       <x:c r="C2" s="1"/>
-      <x:c r="D2" s="1"/>
+      <x:c r="D2" s="1" t="str">
+        <x:v>Treadmills</x:v>
+      </x:c>
       <x:c r="E2" s="1"/>
       <x:c r="F2" s="1"/>
       <x:c r="G2" s="1"/>
@@ -1965,14 +1989,16 @@
       <x:c r="K2" s="1"/>
     </x:row>
     <x:row r="3" ht="35" customHeight="1">
-      <x:c r="A3" s="12" t="str">
+      <x:c r="A3" s="13" t="str">
         <x:v>วิธีนำเข้า</x:v>
       </x:c>
       <x:c r="B3" s="11" t="str">
         <x:v>บันทึกเป็น .xlsx แล้วไปที่คลังสินค้า → นำเข้า Excel</x:v>
       </x:c>
       <x:c r="C3" s="1"/>
-      <x:c r="D3" s="1"/>
+      <x:c r="D3" s="1" t="str">
+        <x:v>Skill Mill</x:v>
+      </x:c>
       <x:c r="E3" s="1"/>
       <x:c r="F3" s="1"/>
       <x:c r="G3" s="1"/>
@@ -1982,14 +2008,16 @@
       <x:c r="K3" s="1"/>
     </x:row>
     <x:row r="4" ht="35" customHeight="1">
-      <x:c r="A4" s="12" t="str">
+      <x:c r="A4" s="13" t="str">
         <x:v>ชีตและหัวตาราง</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
         <x:v>ระบบอ่านเฉพาะชีตแรก เก็บชีตสินค้าไว้ก่อน และคงหัวคอลัมน์ที่แถว 1</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
-      <x:c r="D4" s="1"/>
+      <x:c r="D4" s="1" t="str">
+        <x:v>ClimbMill</x:v>
+      </x:c>
       <x:c r="E4" s="1"/>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -1999,14 +2027,16 @@
       <x:c r="K4" s="1"/>
     </x:row>
     <x:row r="5" ht="35" customHeight="1">
-      <x:c r="A5" s="12" t="str">
+      <x:c r="A5" s="13" t="str">
         <x:v>หนึ่งแถวต่อหนึ่งเครื่อง</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
         <x:v>สินค้ารุ่นเดียวกันหลายเครื่องให้แยกแถว ไม่มีคอลัมน์จำนวน</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
-      <x:c r="D5" s="1"/>
+      <x:c r="D5" s="1" t="str">
+        <x:v>Recumbent Bike</x:v>
+      </x:c>
       <x:c r="E5" s="1"/>
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
@@ -2016,14 +2046,16 @@
       <x:c r="K5" s="1"/>
     </x:row>
     <x:row r="6" ht="35" customHeight="1">
-      <x:c r="A6" s="12" t="str">
+      <x:c r="A6" s="13" t="str">
         <x:v>ช่องบังคับ</x:v>
       </x:c>
       <x:c r="B6" s="11" t="str">
         <x:v>แบรนด์ และ รุ่น ต้องมีข้อมูลทุกแถว</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
-      <x:c r="D6" s="1"/>
+      <x:c r="D6" s="1" t="str">
+        <x:v>Upright Bike</x:v>
+      </x:c>
       <x:c r="E6" s="1"/>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -2033,14 +2065,16 @@
       <x:c r="K6" s="1"/>
     </x:row>
     <x:row r="7" ht="35" customHeight="1">
-      <x:c r="A7" s="12" t="str">
+      <x:c r="A7" s="13" t="str">
         <x:v>SKU</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
         <x:v>เว้นว่างเพื่อสร้างอัตโนมัติ หรือกรอกรหัสที่ไม่ซ้ำในไฟล์และในระบบ</x:v>
       </x:c>
       <x:c r="C7" s="1"/>
-      <x:c r="D7" s="1"/>
+      <x:c r="D7" s="1" t="str">
+        <x:v>Spinning Bike</x:v>
+      </x:c>
       <x:c r="E7" s="1"/>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
@@ -2050,14 +2084,16 @@
       <x:c r="K7" s="1"/>
     </x:row>
     <x:row r="8" ht="35" customHeight="1">
-      <x:c r="A8" s="12" t="str">
+      <x:c r="A8" s="13" t="str">
         <x:v>หมายเลขเครื่อง</x:v>
       </x:c>
       <x:c r="B8" s="11" t="str">
         <x:v>กรอกเป็นข้อความเพื่อรักษาเลขศูนย์นำหน้า เว้นว่างได้</x:v>
       </x:c>
       <x:c r="C8" s="1"/>
-      <x:c r="D8" s="1"/>
+      <x:c r="D8" s="1" t="str">
+        <x:v>Air Bike</x:v>
+      </x:c>
       <x:c r="E8" s="1"/>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -2067,14 +2103,16 @@
       <x:c r="K8" s="1"/>
     </x:row>
     <x:row r="9" ht="35" customHeight="1">
-      <x:c r="A9" s="12" t="str">
+      <x:c r="A9" s="13" t="str">
         <x:v>สภาพ</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
         <x:v>Excellent = ดีเยี่ยม / Good = ดี / Fair = พอใช้ / Needs Repair = ต้องซ่อม</x:v>
       </x:c>
       <x:c r="C9" s="1"/>
-      <x:c r="D9" s="1"/>
+      <x:c r="D9" s="1" t="str">
+        <x:v>Arm Bike</x:v>
+      </x:c>
       <x:c r="E9" s="1"/>
       <x:c r="F9" s="1"/>
       <x:c r="G9" s="1"/>
@@ -2084,14 +2122,16 @@
       <x:c r="K9" s="1"/>
     </x:row>
     <x:row r="10" ht="35" customHeight="1">
-      <x:c r="A10" s="12" t="str">
+      <x:c r="A10" s="13" t="str">
         <x:v>ต้นทุน / ราคาขาย</x:v>
       </x:c>
       <x:c r="B10" s="11" t="str">
         <x:v>หน่วยบาท ตัวเลขตั้งแต่ 0 ถึง 999999999 ทศนิยมไม่เกิน 2 ตำแหน่ง</x:v>
       </x:c>
       <x:c r="C10" s="1"/>
-      <x:c r="D10" s="1"/>
+      <x:c r="D10" s="1" t="str">
+        <x:v>Rowwing</x:v>
+      </x:c>
       <x:c r="E10" s="1"/>
       <x:c r="F10" s="1"/>
       <x:c r="G10" s="1"/>
@@ -2101,14 +2141,16 @@
       <x:c r="K10" s="1"/>
     </x:row>
     <x:row r="11" ht="35" customHeight="1">
-      <x:c r="A11" s="12" t="str">
+      <x:c r="A11" s="13" t="str">
         <x:v>ราคาเมื่อเว้นว่าง</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
         <x:v>ระบบบันทึกเป็น 0 กรุณาตรวจราคาก่อนนำเข้า</x:v>
       </x:c>
       <x:c r="C11" s="1"/>
-      <x:c r="D11" s="1"/>
+      <x:c r="D11" s="1" t="str">
+        <x:v>Elliptical</x:v>
+      </x:c>
       <x:c r="E11" s="1"/>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
@@ -2118,14 +2160,16 @@
       <x:c r="K11" s="1"/>
     </x:row>
     <x:row r="12" ht="35" customHeight="1">
-      <x:c r="A12" s="12" t="str">
+      <x:c r="A12" s="13" t="str">
         <x:v>สถานะ</x:v>
       </x:c>
       <x:c r="B12" s="11" t="str">
         <x:v>พร้อมขาย หรือ ขายแล้ว; เว้นว่างจะเป็นพร้อมขาย</x:v>
       </x:c>
       <x:c r="C12" s="1"/>
-      <x:c r="D12" s="1"/>
+      <x:c r="D12" s="1" t="str">
+        <x:v>Machine Pin</x:v>
+      </x:c>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
@@ -2135,14 +2179,16 @@
       <x:c r="K12" s="1"/>
     </x:row>
     <x:row r="13" ht="35" customHeight="1">
-      <x:c r="A13" s="12" t="str">
+      <x:c r="A13" s="13" t="str">
         <x:v>การจอง</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
         <x:v>นำเข้าเป็นพร้อมขายก่อน แล้วจึงจองให้ลูกค้าจากหน้ารายละเอียดสินค้า</x:v>
       </x:c>
       <x:c r="C13" s="1"/>
-      <x:c r="D13" s="1"/>
+      <x:c r="D13" s="1" t="str">
+        <x:v>Plate Load</x:v>
+      </x:c>
       <x:c r="E13" s="1"/>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
@@ -2152,14 +2198,16 @@
       <x:c r="K13" s="1"/>
     </x:row>
     <x:row r="14" ht="35" customHeight="1">
-      <x:c r="A14" s="12" t="str">
+      <x:c r="A14" s="13" t="str">
         <x:v>รายการขายแล้ว</x:v>
       </x:c>
       <x:c r="B14" s="11" t="str">
         <x:v>ใช้วันที่นำเข้าเป็นวันขาย จึงควรใช้พร้อมขายสำหรับสินค้าคงคลัง</x:v>
       </x:c>
       <x:c r="C14" s="1"/>
-      <x:c r="D14" s="1"/>
+      <x:c r="D14" s="1" t="str">
+        <x:v>Pilatis</x:v>
+      </x:c>
       <x:c r="E14" s="1"/>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
@@ -2169,14 +2217,16 @@
       <x:c r="K14" s="1"/>
     </x:row>
     <x:row r="15" ht="35" customHeight="1">
-      <x:c r="A15" s="12" t="str">
-        <x:v>ช่องอื่น</x:v>
+      <x:c r="A15" s="13" t="str">
+        <x:v>หมวดหมู่</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>หมวดหมู่ สถานที่ และหมายเหตุ เว้นว่างได้</x:v>
+        <x:v>เลือกจาก dropdown 24 หมวดในคอลัมน์ D (แถว 2–201) หรือเว้นว่างได้</x:v>
       </x:c>
       <x:c r="C15" s="1"/>
-      <x:c r="D15" s="1"/>
+      <x:c r="D15" s="1" t="str">
+        <x:v>Dumbbell</x:v>
+      </x:c>
       <x:c r="E15" s="1"/>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
@@ -2186,14 +2236,16 @@
       <x:c r="K15" s="1"/>
     </x:row>
     <x:row r="16" ht="35" customHeight="1">
-      <x:c r="A16" s="12" t="str">
+      <x:c r="A16" s="13" t="str">
         <x:v>ขนาดไฟล์</x:v>
       </x:c>
       <x:c r="B16" s="11" t="str">
         <x:v>สูงสุด 200 รายการต่อไฟล์ และขนาดไม่เกิน 5 MB</x:v>
       </x:c>
       <x:c r="C16" s="1"/>
-      <x:c r="D16" s="1"/>
+      <x:c r="D16" s="1" t="str">
+        <x:v>Dumbbell+Rack</x:v>
+      </x:c>
       <x:c r="E16" s="1"/>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
@@ -2203,14 +2255,16 @@
       <x:c r="K16" s="1"/>
     </x:row>
     <x:row r="17" ht="35" customHeight="1">
-      <x:c r="A17" s="12" t="str">
+      <x:c r="A17" s="13" t="str">
         <x:v>รูปภาพ</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
         <x:v>เพิ่มรูปจากหน้ารายละเอียดสินค้าหลังนำเข้า</x:v>
       </x:c>
       <x:c r="C17" s="1"/>
-      <x:c r="D17" s="1"/>
+      <x:c r="D17" s="1" t="str">
+        <x:v>Barbell+Rack</x:v>
+      </x:c>
       <x:c r="E17" s="1"/>
       <x:c r="F17" s="1"/>
       <x:c r="G17" s="1"/>
@@ -2220,14 +2274,16 @@
       <x:c r="K17" s="1"/>
     </x:row>
     <x:row r="18" ht="35" customHeight="1">
-      <x:c r="A18" s="12" t="str">
+      <x:c r="A18" s="13" t="str">
         <x:v>ตรวจสอบก่อนอัปโหลด</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
         <x:v>ลบแถวตัวอย่างที่ไม่ใช้ ห้ามเพิ่มแถวสรุปยอดหรือคำอธิบายในชีตสินค้า</x:v>
       </x:c>
       <x:c r="C18" s="1"/>
-      <x:c r="D18" s="1"/>
+      <x:c r="D18" s="1" t="str">
+        <x:v>Rack</x:v>
+      </x:c>
       <x:c r="E18" s="1"/>
       <x:c r="F18" s="1"/>
       <x:c r="G18" s="1"/>
@@ -2236,11 +2292,17 @@
       <x:c r="J18" s="1"/>
       <x:c r="K18" s="1"/>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="1"/>
-      <x:c r="B19" s="1"/>
+    <x:row r="19" ht="35" customHeight="1">
+      <x:c r="A19" s="13" t="str">
+        <x:v>หมวดหมู่อื่น</x:v>
+      </x:c>
+      <x:c r="B19" s="11" t="str">
+        <x:v>เลือก Other หากไม่ตรงกับรายการ ห้ามเพิ่มหรือเปลี่ยนรายชื่อหมวดในชีตนี้</x:v>
+      </x:c>
       <x:c r="C19" s="1"/>
-      <x:c r="D19" s="1"/>
+      <x:c r="D19" s="1" t="str">
+        <x:v>Station/Cable/Smith</x:v>
+      </x:c>
       <x:c r="E19" s="1"/>
       <x:c r="F19" s="1"/>
       <x:c r="G19" s="1"/>
@@ -2249,11 +2311,17 @@
       <x:c r="J19" s="1"/>
       <x:c r="K19" s="1"/>
     </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="1"/>
-      <x:c r="B20" s="1"/>
+    <x:row r="20" ht="35" customHeight="1">
+      <x:c r="A20" s="13" t="str">
+        <x:v>การตรวจหมวดหมู่</x:v>
+      </x:c>
+      <x:c r="B20" s="11" t="str">
+        <x:v>ระบบปรับตัวพิมพ์และช่องว่างให้ตรงชื่อมาตรฐาน หมวดไม่ถูกต้องจะแจ้งเลขแถว</x:v>
+      </x:c>
       <x:c r="C20" s="1"/>
-      <x:c r="D20" s="1"/>
+      <x:c r="D20" s="1" t="str">
+        <x:v>Bench</x:v>
+      </x:c>
       <x:c r="E20" s="1"/>
       <x:c r="F20" s="1"/>
       <x:c r="G20" s="1"/>
@@ -2262,6 +2330,43 @@
       <x:c r="J20" s="1"/>
       <x:c r="K20" s="1"/>
     </x:row>
+    <x:row r="21" ht="35" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>ไฟล์เดิม</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>แก้หมวดเดิม เช่น ลู่วิ่ง → Treadmills ให้ตรงรายการก่อนนำเข้า</x:v>
+      </x:c>
+      <x:c r="D21" s="1" t="str">
+        <x:v>Accessories</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="35" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>เมื่อพบข้อผิดพลาด</x:v>
+      </x:c>
+      <x:c r="B22" s="12" t="str">
+        <x:v>แก้ทุกแถวที่แจ้งแล้วนำเข้าใหม่ ระบบยังไม่เพิ่มสินค้าใดจนกว่าทุกแถวจะผ่าน</x:v>
+      </x:c>
+      <x:c r="D22" s="1" t="str">
+        <x:v>Plate</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="35" customHeight="1">
+      <x:c r="D23" s="1" t="str">
+        <x:v>Ski</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="35" customHeight="1">
+      <x:c r="D24" s="1" t="str">
+        <x:v>Stepper</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="35" customHeight="1">
+      <x:c r="D25" s="1" t="str">
+        <x:v>Other</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>